<commit_message>
Add AI MCQ banks and refresh the Python question workbooks
300 AI questions, 50 per unit, in markdown alongside the upload workbooks.
The first 20 of each unit cover every subtopic and form Set 1 for the course;
the remaining 30 are Set 2, held in reserve.

Answer keys are shuffled rather than cycled, so no ascending run of options
and no distractor position dominates. Explanations name distractors by their
content instead of by option number, which keeps them valid under reshuffling.

Also drops the .bak files and one-shot build scripts from the DBMS and Python
banks, whose generated workbooks are what matters, and updates the Python
workbooks to their current content.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Python/Unit 11 - File Handling/Unit 11 - File Handling - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Python/Unit 11 - File Handling/Unit 11 - File Handling - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 11" sheetId="1" r:id="R4d5a91fcc0c84828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 11" sheetId="1" r:id="R95d6be2d6fdb43f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -405,15 +405,17 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="18" customHeight="1">
+    <x:row r="2" ht="60" hidden="0" customHeight="1">
       <x:c r="A2" s="1" t="str">
         <x:v>Python - MCQ - 11.1.1</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
-        <x:v>A game keeps the player's score only in a variable. Every restart resets it to zero. Which change gives the score persistence?</x:v>
+        <x:v>Make a score survive the end of the program
+A game stores the current score in a variable, but the score disappears whenever the program closes. The next run must recover the previous value.
+Which change provides persistence?</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>Variables live only while a program runs. Writing the score to a file places it on disk so a later run can read it back.</x:v>
+        <x:v>File data remains on disk after the process ends, while ordinary variables exist only during execution.</x:v>
       </x:c>
       <x:c r="D2" s="4" t="n">
         <x:v>1</x:v>
@@ -425,7 +427,7 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>understand</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H2" s="1" t="str">
         <x:v>python - Set 1</x:v>
@@ -441,30 +443,32 @@
       </x:c>
       <x:c r="L2" s="1"/>
       <x:c r="M2" s="1" t="str">
-        <x:v>Keep the program continuously running so its memory is never released</x:v>
+        <x:v>Assign the score to a second variable before exiting.</x:v>
       </x:c>
       <x:c r="N2" s="1" t="str">
-        <x:v>Write the score to a file and read it on the next run</x:v>
+        <x:v>Persist the score in a file and reload it.</x:v>
       </x:c>
       <x:c r="O2" s="1" t="str">
-        <x:v>Rename the score variable</x:v>
+        <x:v>Print the score twice before closing.</x:v>
       </x:c>
       <x:c r="P2" s="1" t="str">
-        <x:v>Place the score inside a loop</x:v>
+        <x:v>Store the score in a loop variable.</x:v>
       </x:c>
       <x:c r="Q2" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="18" customHeight="1">
+    <x:row r="3" ht="60" hidden="0" customHeight="1">
       <x:c r="A3" s="1" t="str">
         <x:v>Python - MCQ - 11.1.2</x:v>
       </x:c>
       <x:c r="B3" s="1" t="str">
-        <x:v>A report should be written and closed automatically when its block ends. Which opening statement has the correct structure?</x:v>
+        <x:v>Choose the read shape required by a validator
+A validator must compare every saved wristband line by line and also retain all lines as a list for later indexing.
+Which reading operation directly returns that required list shape?</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>`with open(...) as file:` creates a context-managed file. Python closes it when the indented block ends, even if the block exits because of an error.</x:v>
+        <x:v>`readlines()` returns a list containing one string per line, including stored line endings.</x:v>
       </x:c>
       <x:c r="D3" s="4" t="n">
         <x:v>1</x:v>
@@ -473,10 +477,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F3" s="1" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G3" s="2" t="str">
-        <x:v>apply</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H3" s="1" t="str">
         <x:v>python - Set 1</x:v>
@@ -488,34 +492,44 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K3" s="1" t="str">
-        <x:v>context-managed-files</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L3" s="1"/>
       <x:c r="M3" s="1" t="str">
-        <x:v>`open with 'report.txt' as file:`</x:v>
+        <x:v>`file.write("all lines")`</x:v>
       </x:c>
       <x:c r="N3" s="1" t="str">
-        <x:v>`with file = open('report.txt', 'w'):`</x:v>
+        <x:v>`file.read()`</x:v>
       </x:c>
       <x:c r="O3" s="1" t="str">
-        <x:v>`using open('report.txt', 'w') as file:`</x:v>
+        <x:v>`file.close()`</x:v>
       </x:c>
       <x:c r="P3" s="1" t="str">
-        <x:v>`with open('report.txt', 'w') as file:`</x:v>
+        <x:v>`file.readlines()`</x:v>
       </x:c>
       <x:c r="Q3" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="198" hidden="0" customHeight="1">
       <x:c r="A4" t="str">
         <x:v>Python - MCQ - 11.1.3</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>A reports folder contains CSV, TXT, and JSON files. Which glob pattern selects every CSV file directly inside that folder?</x:v>
+        <x:v>Trace two file modes applied in sequence
+A daily log already contains `OLD
+`. A reset step is followed by two new scans.
+```python
+with open("log.txt", "w", encoding="utf-8") as file:
+    file.write("A101\n")
+with open("log.txt", "a", encoding="utf-8") as file:
+    file.write("A102\n")
+    file.write("A103\n")
+```
+Which final content should the audit expect?</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>The `*` wildcard matches any filename portion within one folder level. `*.csv` therefore selects filenames ending in `.csv`.</x:v>
+        <x:v>The first open in write mode erases the old content; append mode then preserves A101 and adds two lines.</x:v>
       </x:c>
       <x:c r="D4" t="n">
         <x:v>1</x:v>
@@ -524,7 +538,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>easy</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G4" t="str">
         <x:v>apply</x:v>
@@ -539,42 +553,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>glob-pattern-matching</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L4"/>
       <x:c r="M4" t="str">
-        <x:v>`*.csv`</x:v>
+        <x:v>`A101\nA102\nA103\n`</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>`**.txt`</x:v>
+        <x:v>`OLD\nA101\nA102\nA103\n`</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>`csv.*`</x:v>
+        <x:v>`A103\n`</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>`*.json`</x:v>
+        <x:v>`OLD\nA102\nA103\n`</x:v>
       </x:c>
       <x:c r="Q4" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
       <x:c r="A5" t="str">
         <x:v>Python - MCQ - 11.1.4</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>A scanner writes two IDs and reads them as separate lines.
-```python
-with open('ids.txt', 'w') as file:
-    file.write('A1\nA2\n')
-with open('ids.txt', 'r') as file:
-    lines = file.readlines()
-print(lines)
-```
-What is displayed?</x:v>
+        <x:v>Guarantee closure when processing fails
+A report may encounter a calculation failure after opening a file. The file must still be closed when control leaves the writing block.
+Which structure supplies that guarantee?</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>`readlines()` returns one string per line and keeps each trailing newline. Both saved lines therefore include `\n` in the list representation.</x:v>
+        <x:v>A `with` block releases the file whether the block completes normally or exits because of an error.</x:v>
       </x:c>
       <x:c r="D5" t="n">
         <x:v>1</x:v>
@@ -586,7 +594,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>python - Set 1</x:v>
@@ -598,34 +606,41 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>context-managed-files</x:v>
       </x:c>
       <x:c r="L5"/>
       <x:c r="M5" t="str">
-        <x:v>`['A1', 'A2']`</x:v>
+        <x:v>Open the file globally and never close it.</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>`'A1\nA2\n'` returned as one string</x:v>
+        <x:v>Put `file.close()` after the line that may terminate execution.</x:v>
       </x:c>
       <x:c r="O5" t="str">
-        <x:v>`['A1\n', 'A2\n']`</x:v>
+        <x:v>Use `with open(...) as file:` for the file operation.</x:v>
       </x:c>
       <x:c r="P5" t="str">
-        <x:v>`[A1, A2]`</x:v>
+        <x:v>Open the same file a second time after the calculation.</x:v>
       </x:c>
       <x:c r="Q5" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A6" t="str">
         <x:v>Python - MCQ - 11.1.5</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>A script must build a cross-platform path to `reports/day1.txt` without manually inserting a slash. Which expression is appropriate?</x:v>
+        <x:v>Build a path without guessing the operating system's separator
+A report must be stored as `reports/daily.txt` on Windows, macOS, and Linux without manually concatenating slashes.
+```python
+from pathlib import Path
+folder = Path("reports")
+report = ________
+```
+Which expression completes the path safely?</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>`Path('reports') / 'day1.txt'` joins path components using `pathlib`, which handles operating-system path details.</x:v>
+        <x:v>`Path` uses `/` to join path components correctly for the current operating system.</x:v>
       </x:c>
       <x:c r="D6" t="n">
         <x:v>1</x:v>
@@ -653,30 +668,32 @@
       </x:c>
       <x:c r="L6"/>
       <x:c r="M6" t="str">
-        <x:v>`Path('reports').split('day1.txt')`</x:v>
+        <x:v>`folder / "daily.txt"`</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>`Path('reports') / 'day1.txt'`</x:v>
+        <x:v>`folder.divide("daily.txt")`</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>`Path('reports') + Path('day1.txt')`</x:v>
+        <x:v>`folder + "/" + "daily.txt"`</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>`open('reports') / 'day1.txt'`</x:v>
+        <x:v>`"reports" * "daily.txt"`</x:v>
       </x:c>
       <x:c r="Q6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="66" hidden="0" customHeight="1">
       <x:c r="A7" t="str">
         <x:v>Python - MCQ - 11.1.6</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>A sales CSV has headers `item,quantity,price`. The code should read `row['quantity']` instead of remembering that quantity is column 1. Which reader supports that design?</x:v>
+        <x:v>Select all CSV files in one reports folder
+A reports folder contains several file types. A script needs every filename ending in `.csv` directly inside that folder.
+Which pattern describes that set?</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>`csv.DictReader` uses the header row as dictionary keys. Each data row can then be accessed by meaningful column names.</x:v>
+        <x:v>`*` matches any filename characters within the current folder, followed by the required `.csv` suffix.</x:v>
       </x:c>
       <x:c r="D7" t="n">
         <x:v>1</x:v>
@@ -685,10 +702,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H7" t="str">
         <x:v>python - Set 1</x:v>
@@ -700,34 +717,40 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>csv-processing</x:v>
+        <x:v>glob-pattern-matching</x:v>
       </x:c>
       <x:c r="L7"/>
       <x:c r="M7" t="str">
-        <x:v>`csv.DictReader(file)`</x:v>
+        <x:v>`**.txt`</x:v>
       </x:c>
       <x:c r="N7" t="str">
-        <x:v>`file.readlines()`</x:v>
+        <x:v>`csv.*`</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>`csv.writer(file)`</x:v>
+        <x:v>`*.csv`</x:v>
       </x:c>
       <x:c r="P7" t="str">
-        <x:v>`json.load(file)` with automatic CSV header mapping</x:v>
+        <x:v>`csv`</x:v>
       </x:c>
       <x:c r="Q7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="132" hidden="0" customHeight="1">
       <x:c r="A8" t="str">
         <x:v>Python - MCQ - 11.1.7</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>A fest report contains dictionaries nested inside dictionaries. Why is JSON a better storage choice than CSV for this data?</x:v>
+        <x:v>Correct arithmetic performed on CSV text
+A sales calculation reads quantity and price with `csv.DictReader`. The row looks numeric in the file, but multiplication does not behave as intended because CSV values arrive as text.
+```python
+row = {"item": "Mug", "quantity": "2", "price": "150"}
+total = row["quantity"] * row["price"]
+```
+Which smallest repair produces numeric `300`?</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>JSON represents nested dictionaries and lists directly. CSV is naturally flat and table-shaped, so it cannot preserve the same nested structure cleanly.</x:v>
+        <x:v>Each CSV field must be converted separately from text to an integer before arithmetic.</x:v>
       </x:c>
       <x:c r="D8" t="n">
         <x:v>1</x:v>
@@ -736,7 +759,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G8" t="str">
         <x:v>analyze</x:v>
@@ -751,34 +774,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>json-processing</x:v>
+        <x:v>csv-processing</x:v>
       </x:c>
       <x:c r="L8"/>
       <x:c r="M8" t="str">
-        <x:v>CSV cannot store any text</x:v>
+        <x:v>`total = str(row["quantity"]) * str(row["price"])`</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>JSON automatically encrypts every value</x:v>
+        <x:v>`total = row["quantity"] + row["price"]`</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>CSV always converts numbers to zero</x:v>
+        <x:v>`total = int(row["quantity"] * row["price"])`</x:v>
       </x:c>
       <x:c r="P8" t="str">
-        <x:v>JSON naturally preserves nested data structures</x:v>
+        <x:v>`total = int(row["quantity"]) * int(row["price"])`</x:v>
       </x:c>
       <x:c r="Q8" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
       <x:c r="A9" t="str">
         <x:v>Python - MCQ - 11.1.8</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>`attendees.txt` already contains 80 IDs. A registration script opens it with mode `'w'` before writing one new ID. What is the consequence?</x:v>
+        <x:v>Preserve a nested stall report across runs
+A report is a dictionary whose stall names map to inner item-price dictionaries. It must be saved and restored with its nesting intact.
+Which format and module best match that shape?</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Write mode truncates an existing file immediately. The previous IDs are erased, and the file contains only what the new session writes.</x:v>
+        <x:v>JSON naturally represents nested dictionaries and lists and reconstructs them as Python structures.</x:v>
       </x:c>
       <x:c r="D9" t="n">
         <x:v>1</x:v>
@@ -787,10 +812,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H9" t="str">
         <x:v>python - Set 1</x:v>
@@ -802,41 +827,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L9"/>
       <x:c r="M9" t="str">
-        <x:v>The new ID is rejected</x:v>
+        <x:v>Plain text with manual string splitting</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>The old and new IDs are merged automatically</x:v>
+        <x:v>JSON using Python's `json` module</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>The existing content is erased before the new write</x:v>
+        <x:v>CSV with one unlabelled cell</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Python changes the mode to append</x:v>
+        <x:v>A variable that is never written to disk</x:v>
       </x:c>
       <x:c r="Q9" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="66" hidden="0" customHeight="1">
       <x:c r="A10" t="str">
         <x:v>Python - MCQ - 11.1.9</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>A report crashes inside a managed file block.
-```python
-with open('report.txt', 'w') as file:
-    file.write('Line 1\n')
-    value = 10 / 0
-    file.write('Line 2\n')
-```
-Which statement describes the file state?</x:v>
+        <x:v>Defend a read and preserve a rupee symbol
+A receipt file may not exist on a teammate's machine, and when it does exist it can contain `₹`. Unit 12 exception handling is not yet available.
+Which approach addresses both risks using only Unit 11 tools?</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>The division raises `ZeroDivisionError`, so the second write never runs. The context manager still closes the file, preserving the first line written before the failure.</x:v>
+        <x:v>The existence guard prevents a missing-file read, while explicit UTF-8 keeps character interpretation consistent.</x:v>
       </x:c>
       <x:c r="D10" t="n">
         <x:v>1</x:v>
@@ -860,34 +880,41 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>context-managed-files</x:v>
+        <x:v>file-errors</x:v>
       </x:c>
       <x:c r="L10"/>
       <x:c r="M10" t="str">
-        <x:v>Both lines are written before the error appears</x:v>
+        <x:v>Check existence before reading and use UTF-8 explicitly.</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>The file is closed and contains only Line 1</x:v>
+        <x:v>Open blindly in write mode so a missing file is replaced.</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>The file remains open with both lines</x:v>
+        <x:v>Remove every non-English character before saving.</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>The file is deleted automatically</x:v>
+        <x:v>Use `readlines()` without checking the path or encoding.</x:v>
       </x:c>
       <x:c r="Q10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A11" t="str">
         <x:v>Python - MCQ - 11.1.10</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>A receipt reader must avoid crashing when a file is absent and must preserve a rupee symbol across different machines. Which approach addresses both risks within this unit's scope?</x:v>
+        <x:v>Keep individual lines clean while streaming a large file
+A very large attendee file should be processed one line at a time rather than loaded fully into memory. Stored newline characters must not remain in the IDs.
+```python
+with open("attendees.txt", "r", encoding="utf-8") as file:
+    for line in file:
+        attendee_id = ________
+```
+Which expression completes the cleanup?</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>`Path.exists()` can guard the read before opening a missing file, while explicit UTF-8 on both writes and reads keeps character interpretation consistent.</x:v>
+        <x:v>Direct iteration streams one line at a time, and `rstrip("\r\n")` removes line-ending characters without deleting meaningful spaces elsewhere in the ID.</x:v>
       </x:c>
       <x:c r="D11" t="n">
         <x:v>1</x:v>
@@ -896,10 +923,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H11" t="str">
         <x:v>python - Set 1</x:v>
@@ -911,34 +938,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>file-errors</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L11"/>
       <x:c r="M11" t="str">
-        <x:v>Check `Path.exists()` first and use `encoding='utf-8'` consistently</x:v>
+        <x:v>`line.lstrip()`</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>Use write mode for every read</x:v>
+        <x:v>`line.replace(" ", "")`</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>Remove all non-English characters</x:v>
+        <x:v>`line.rstrip("\r\n")`</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>Assume every machine uses the same default encoding</x:v>
+        <x:v>`line.split(",")`</x:v>
       </x:c>
       <x:c r="Q11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66" hidden="0" customHeight="1">
       <x:c r="A12" t="str">
         <x:v>Python - MCQ - 11.2.1</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>A developer needs the complete contents of a small text file as one string. Which file method directly provides that shape?</x:v>
+        <x:v>Put separate IDs on separate lines
+A wristband logger writes one ID per call. The file currently stores `A101A102` on one line because `write()` adds no separator automatically.
+Which write preserves the intended line structure?</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>`read()` returns the entire remaining file contents as one string, including any embedded newline characters.</x:v>
+        <x:v>The newline must be included explicitly in the string passed to `write()`.</x:v>
       </x:c>
       <x:c r="D12" t="n">
         <x:v>1</x:v>
@@ -950,7 +979,7 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H12" t="str">
         <x:v>python - Set 2</x:v>
@@ -966,30 +995,32 @@
       </x:c>
       <x:c r="L12"/>
       <x:c r="M12" t="str">
-        <x:v>`writelines()`</x:v>
+        <x:v>`file.write("A103")`</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>`readlines()`</x:v>
+        <x:v>`file.writelines(["A103"])`</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>`read()`</x:v>
+        <x:v>`file.write("A103" + "")`</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>`write()`</x:v>
+        <x:v>`file.write("A103\n")`</x:v>
       </x:c>
       <x:c r="Q12" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="66" hidden="0" customHeight="1">
       <x:c r="A13" t="str">
         <x:v>Python - MCQ - 11.2.2</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>A multi-gigabyte log should be processed without loading every line into a list first. Which pattern is most memory-efficient?</x:v>
+        <x:v>Process a huge log without constructing a list of every line
+A multi-gigabyte log needs one validation check per line, and no later step needs all lines in memory together.
+Which approach is most appropriate?</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>Looping directly over the open file yields one line at a time. It avoids storing the entire file or a full list of lines in memory.</x:v>
+        <x:v>Direct iteration reads incrementally and avoids storing the entire file or line list at once.</x:v>
       </x:c>
       <x:c r="D13" t="n">
         <x:v>1</x:v>
@@ -998,10 +1029,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H13" t="str">
         <x:v>python - Set 2</x:v>
@@ -1017,30 +1048,32 @@
       </x:c>
       <x:c r="L13"/>
       <x:c r="M13" t="str">
-        <x:v>Call `read()` twice</x:v>
+        <x:v>Call `read()` and split the resulting whole-file string.</x:v>
       </x:c>
       <x:c r="N13" t="str">
-        <x:v>Call `readlines()` before the loop</x:v>
+        <x:v>Loop directly over the open file object.</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>Convert the file to JSON first</x:v>
+        <x:v>Call `readlines()` before beginning the loop.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>Use `for line in file:`</x:v>
+        <x:v>Open the file in append mode.</x:v>
       </x:c>
       <x:c r="Q13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="66" hidden="0" customHeight="1">
       <x:c r="A14" t="str">
         <x:v>Python - MCQ - 11.2.3</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>A file loop receives the line `'A101\n'`, but the ID must be compared as `'A101'`. Which expression removes the surrounding whitespace?</x:v>
+        <x:v>Repair a `writelines` call that merges records
+A batch save uses `writelines(["A101", "A102", "A103"])`, producing one run-together line.
+Which replacement preserves one ID per line?</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>`line.strip()` removes leading and trailing whitespace, including the newline at the end of a file line.</x:v>
+        <x:v>Like `write`, `writelines` adds no line separators; each supplied string must contain its own newline.</x:v>
       </x:c>
       <x:c r="D14" t="n">
         <x:v>1</x:v>
@@ -1052,7 +1085,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H14" t="str">
         <x:v>python - Set 2</x:v>
@@ -1068,30 +1101,32 @@
       </x:c>
       <x:c r="L14"/>
       <x:c r="M14" t="str">
-        <x:v>`line.strip()`</x:v>
+        <x:v>`file.writelines("A101", "A102", "A103")`</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>`line.append()`</x:v>
+        <x:v>`file.writelines(["A101", "A102", "A103"], separator="\n")`</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>`line.readlines()`</x:v>
+        <x:v>`file.writelines(["A101\n", "A102\n", "A103\n"])`</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>`line.close()`</x:v>
+        <x:v>`file.readlines(["A101", "A102", "A103"])`</x:v>
       </x:c>
       <x:c r="Q14" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66" hidden="0" customHeight="1">
       <x:c r="A15" t="str">
         <x:v>Python - MCQ - 11.2.4</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>A writer calls `file.write('A1')` followed by `file.write('A2')`. No newline characters are supplied. What text is stored?</x:v>
+        <x:v>Identify the mode that quietly destroys earlier records
+`audit.txt` initially contains three records. A function intended to add a fourth opens the file with mode `"w"` and writes one new line.
+Which diagnosis and smallest repair are both correct?</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>`write()` adds no separator or line break automatically. The two strings are written consecutively as `A1A2`.</x:v>
+        <x:v>`"w"` empties an existing file on open, whereas `"a"` keeps its contents and writes at the end.</x:v>
       </x:c>
       <x:c r="D15" t="n">
         <x:v>1</x:v>
@@ -1100,10 +1135,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H15" t="str">
         <x:v>python - Set 2</x:v>
@@ -1119,30 +1154,37 @@
       </x:c>
       <x:c r="L15"/>
       <x:c r="M15" t="str">
-        <x:v>A1 and A2 on separate lines</x:v>
+        <x:v>`"w"` truncates the file; change the mode to `"a"`.</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>`A1A2`</x:v>
+        <x:v>Write mode preserves old lines; the defect is a missing `read()`.</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>Only A2</x:v>
+        <x:v>Append mode would delete the file, so use read mode.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>`A1 A2` with an automatic space</x:v>
+        <x:v>All three modes behave identically when the file exists.</x:v>
       </x:c>
       <x:c r="Q15" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A16" t="str">
         <x:v>Python - MCQ - 11.2.5</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>A developer uses `file.writelines(['A1', 'A2', 'A3'])` and expects three lines. Why do the values run together?</x:v>
+        <x:v>Verify the resource state after a normal `with` block
+A test checks whether a file object has been released immediately after the indented `with` block ends.
+```python
+with open("report.txt", "w", encoding="utf-8") as file:
+    file.write("Ready")
+closed_state = file.closed
+```
+Which value is stored in `closed_state`?</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>`writelines()` writes the supplied strings in sequence but does not insert newline characters. Each list element must already contain its required `\n`.</x:v>
+        <x:v>The object name remains accessible, but its managed file resource has already been closed.</x:v>
       </x:c>
       <x:c r="D16" t="n">
         <x:v>1</x:v>
@@ -1154,7 +1196,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H16" t="str">
         <x:v>python - Set 2</x:v>
@@ -1166,34 +1208,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>context-managed-files</x:v>
       </x:c>
       <x:c r="L16"/>
       <x:c r="M16" t="str">
-        <x:v>The list must contain integers</x:v>
+        <x:v>`False`, until `file.close()` is called manually</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>`writelines()` accepts only one value</x:v>
+        <x:v>`True`; leaving the `with` block closes the file</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>Append mode disables line breaks</x:v>
+        <x:v>`None`, because `closed` is a method</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>The strings do not include their own newline characters</x:v>
+        <x:v>The name `file` is deleted when the block ends</x:v>
       </x:c>
       <x:c r="Q16" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66" hidden="0" customHeight="1">
       <x:c r="A17" t="str">
         <x:v>Python - MCQ - 11.2.6</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>A log starts with `Gate open\n`. The script then opens it in append mode and writes `First scan\n`. What remains in the file?</x:v>
+        <x:v>Create a report path from folder and filename objects
+A script already imports `Path` and wants a portable path object for `reports/summary.txt`.
+Which expression creates it directly?</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Append mode preserves existing content and adds new text at the end. Both log entries remain in their original order.</x:v>
+        <x:v>A `Path` object supports `/` for portable component joining.</x:v>
       </x:c>
       <x:c r="D17" t="n">
         <x:v>1</x:v>
@@ -1202,10 +1246,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>apply</x:v>
+        <x:v>understand</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>python - Set 2</x:v>
@@ -1217,34 +1261,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>file-paths</x:v>
       </x:c>
       <x:c r="L17"/>
       <x:c r="M17" t="str">
-        <x:v>Only `First scan`</x:v>
+        <x:v>`Path.join("reports", "summary.txt")`</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>An empty file</x:v>
+        <x:v>`"reports" / "summary.txt"`</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>`Gate open` followed by `First scan`</x:v>
+        <x:v>`Path("reports") + Path("summary.txt")`</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Only `Gate open`</x:v>
+        <x:v>`Path("reports") / "summary.txt"`</x:v>
       </x:c>
       <x:c r="Q17" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66" hidden="0" customHeight="1">
       <x:c r="A18" t="str">
         <x:v>Python - MCQ - 11.2.7</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>An existing report contains important data. A script executes `file = open('report.txt', 'w')` but crashes before calling `write`. What happened to the old content?</x:v>
+        <x:v>Extract filename details without splitting strings
+A classifier receives `Path("reports/day1_sales.csv")` and needs the full filename, base name, and extension.
+Which triple is correct for `(path.name, path.stem, path.suffix)`?</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>Opening an existing file in write mode truncates it immediately. The old content is already gone even though no new write completed.</x:v>
+        <x:v>`name` includes the extension, `stem` removes it, and `suffix` includes the leading dot.</x:v>
       </x:c>
       <x:c r="D18" t="n">
         <x:v>1</x:v>
@@ -1256,7 +1302,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H18" t="str">
         <x:v>python - Set 2</x:v>
@@ -1268,34 +1314,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>file-paths</x:v>
       </x:c>
       <x:c r="L18"/>
       <x:c r="M18" t="str">
-        <x:v>It remains until the first successful write</x:v>
+        <x:v>`("day1_sales.csv", "day1_sales", ".csv")`</x:v>
       </x:c>
       <x:c r="N18" t="str">
-        <x:v>It is erased when the file opens in write mode</x:v>
+        <x:v>`("reports", "day1_sales.csv", "csv")`</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>It moves to a backup file</x:v>
+        <x:v>`("day1_sales", ".csv", "reports")`</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>Python silently switches to read mode</x:v>
+        <x:v>`("reports/day1_sales.csv", "reports", "day1_sales")`</x:v>
       </x:c>
       <x:c r="Q18" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="66" hidden="0" customHeight="1">
       <x:c r="A19" t="str">
         <x:v>Python - MCQ - 11.2.8</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>Why is `with open(...) as file:` preferred over a manual `open()` and later `close()` pair?</x:v>
+        <x:v>Complete a recursive search without changing result types
+Existing code expects `Path` objects and currently uses `reports.glob("*.txt")`, which misses text files in deeper folders. The replacement must remain a `pathlib` operation and search every depth.
+Which replacement satisfies both requirements?</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>The context manager closes the file whenever the block exits, including error paths where a later manual `close()` would never be reached.</x:v>
+        <x:v>`Path.rglob("*.txt")` searches recursively and continues yielding `Path` objects, preserving the interface expected by later code.</x:v>
       </x:c>
       <x:c r="D19" t="n">
         <x:v>1</x:v>
@@ -1304,10 +1352,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>python - Set 2</x:v>
@@ -1319,40 +1367,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>context-managed-files</x:v>
+        <x:v>glob-pattern-matching</x:v>
       </x:c>
       <x:c r="L19"/>
       <x:c r="M19" t="str">
-        <x:v>It guarantees the file is closed when the block exits</x:v>
+        <x:v>`glob.glob("reports/**/*.txt")` without enabling recursive matching</x:v>
       </x:c>
       <x:c r="N19" t="str">
-        <x:v>It makes every file read-only</x:v>
+        <x:v>`reports.glob("*.txt")` followed by converting each result to a string</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>It prevents all runtime errors</x:v>
+        <x:v>`reports.rglob("*.txt")`</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>It automatically converts text to CSV</x:v>
+        <x:v>`reports.iterdir()` with no traversal of child folders</x:v>
       </x:c>
       <x:c r="Q19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="66" hidden="0" customHeight="1">
       <x:c r="A20" t="str">
         <x:v>Python - MCQ - 11.2.9</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>A script checks a file object immediately after its `with` block.
-```python
-with open('note.txt', 'w') as file:
-    file.write('saved')
-print(file.closed)
-```
-What is printed?</x:v>
+        <x:v>Read named CSV columns without memorising positions
+A sales file has headers `item,quantity,price`, and the processing code should use expressions such as `row["price"]`.
+Which reader supplies each row in that form?</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>The context manager closes the file as soon as the indented block ends. Its `closed` attribute is therefore `True`.</x:v>
+        <x:v>`DictReader` uses the header row as keys and returns each data row as a dictionary.</x:v>
       </x:c>
       <x:c r="D20" t="n">
         <x:v>1</x:v>
@@ -1364,7 +1408,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>apply</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>python - Set 2</x:v>
@@ -1376,34 +1420,42 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K20" t="str">
-        <x:v>context-managed-files</x:v>
+        <x:v>csv-processing</x:v>
       </x:c>
       <x:c r="L20"/>
       <x:c r="M20" t="str">
-        <x:v>saved</x:v>
+        <x:v>`csv.reader(file)`</x:v>
       </x:c>
       <x:c r="N20" t="str">
-        <x:v>False</x:v>
+        <x:v>`csv.DictReader(file)`</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>True</x:v>
+        <x:v>`csv.DictWriter(file, fieldnames=...)`</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>None</x:v>
+        <x:v>`csv.writer(file)`</x:v>
       </x:c>
       <x:c r="Q20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A21" t="str">
         <x:v>Python - MCQ - 11.2.10</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>For `Path('reports/day1_sales.csv')`, which property returns only `.csv`?</x:v>
+        <x:v>Complete a CSV export with a header and ordered fields
+A list of sale dictionaries must become a CSV with columns ordered as `item`, `quantity`, and `price`, including one header row.
+```python
+fieldnames = ["item", "quantity", "price"]
+writer = csv.DictWriter(file, fieldnames=fieldnames)
+________
+writer.writerows(sales)
+```
+Which missing line produces the required header exactly once?</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>A Path object's `.suffix` property returns the final file extension including its leading dot.</x:v>
+        <x:v>`writeheader()` writes the configured field names as the CSV header before the data rows.</x:v>
       </x:c>
       <x:c r="D21" t="n">
         <x:v>1</x:v>
@@ -1412,7 +1464,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G21" t="str">
         <x:v>apply</x:v>
@@ -1427,34 +1479,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K21" t="str">
-        <x:v>file-paths</x:v>
+        <x:v>csv-processing</x:v>
       </x:c>
       <x:c r="L21"/>
       <x:c r="M21" t="str">
-        <x:v>`.name`</x:v>
+        <x:v>`writer.writerow(fieldnames)`</x:v>
       </x:c>
       <x:c r="N21" t="str">
-        <x:v>The `.stem` property without an extension</x:v>
+        <x:v>`writer.writerows(sales)`</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>`.parent`</x:v>
+        <x:v>`writer.writerow(sales[0])`</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>`.suffix`</x:v>
+        <x:v>`writer.writeheader()`</x:v>
       </x:c>
       <x:c r="Q21" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="66" hidden="0" customHeight="1">
       <x:c r="A22" t="str">
         <x:v>Python - MCQ - 11.3.1</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>A report path should be assembled from a folder object and a filename. Which `pathlib` expression is correct?</x:v>
+        <x:v>Convert a Python structure to JSON text in memory
+An application needs JSON text to send elsewhere, but it does not want to open a file.
+Which function returns a JSON string?</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>Path objects use `/` to join path components safely. The result points to `reports/summary.txt` using the current platform's path rules.</x:v>
+        <x:v>The `s` in `dumps` indicates conversion from a Python object to a JSON string.</x:v>
       </x:c>
       <x:c r="D22" t="n">
         <x:v>1</x:v>
@@ -1463,10 +1517,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>apply</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>python - Set 3</x:v>
@@ -1478,34 +1532,41 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K22" t="str">
-        <x:v>file-paths</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L22"/>
       <x:c r="M22" t="str">
-        <x:v>`Path('reports') / 'summary.txt'`</x:v>
+        <x:v>`json.dump(data, file)`</x:v>
       </x:c>
       <x:c r="N22" t="str">
-        <x:v>`Path('reports').append('summary.txt')`</x:v>
+        <x:v>`json.load(file)`</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>`Path('reports') * 'summary.txt'`</x:v>
+        <x:v>`json.dumps(data)`</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>`'reports'.Path('summary.txt')`</x:v>
+        <x:v>`json.loads(data)`</x:v>
       </x:c>
       <x:c r="Q22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A23" t="str">
         <x:v>Python - MCQ - 11.3.2</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>A setup command may run repeatedly, but it should create `reports` only when needed and not fail if it already exists. Which call fits?</x:v>
+        <x:v>Account for a tuple after a JSON round trip
+A location is stored as a Python tuple, converted to JSON text, and then loaded back. The program must know whether tuple identity survives.
+```python
+import json
+original = {"location": (15.2, 74.1)}
+restored = json.loads(json.dumps(original))
+```
+Which value and type does `restored["location"]` have?</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>`Path('reports').mkdir(exist_ok=True)` creates the folder and suppresses the already-exists error on later runs.</x:v>
+        <x:v>JSON represents both Python lists and tuples as arrays, which load back into Python as lists.</x:v>
       </x:c>
       <x:c r="D23" t="n">
         <x:v>1</x:v>
@@ -1517,7 +1578,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H23" t="str">
         <x:v>python - Set 3</x:v>
@@ -1529,34 +1590,40 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>file-paths</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L23"/>
       <x:c r="M23" t="str">
-        <x:v>`Path('reports').write_text('create the folder now')`</x:v>
+        <x:v>`[15.2, 74.1]`, a list</x:v>
       </x:c>
       <x:c r="N23" t="str">
-        <x:v>`Path('reports').exists(False)`</x:v>
+        <x:v>`(15.2, 74.1)`, a tuple</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>`Path('reports').mkdir(exist_ok=True)`</x:v>
+        <x:v>`"(15.2, 74.1)"`, a string</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>`open('reports', 'a')`</x:v>
+        <x:v>`None`</x:v>
       </x:c>
       <x:c r="Q23" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="132" hidden="0" customHeight="1">
       <x:c r="A24" t="str">
         <x:v>Python - MCQ - 11.3.3</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>A small text file should be overwritten and then read back using only its Path object. Which method pair performs those whole-file operations?</x:v>
+        <x:v>Repair confusion between a JSON file and a JSON string
+A configuration file is already open, but the code passes that file object to the function intended for a string.
+```python
+with open("config.json", "r", encoding="utf-8") as file:
+    config = json.loads(file)
+```
+Which smallest repair uses the open file correctly?</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>`write_text()` writes the entire text content, and `read_text()` reads the entire file back. Both are convenient Path methods for small text files.</x:v>
+        <x:v>`load` reads JSON from an open file; `loads` parses JSON text held in a string.</x:v>
       </x:c>
       <x:c r="D24" t="n">
         <x:v>1</x:v>
@@ -1565,10 +1632,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F24" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>apply</x:v>
+        <x:v>analyze</x:v>
       </x:c>
       <x:c r="H24" t="str">
         <x:v>python - Set 3</x:v>
@@ -1580,34 +1647,42 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>file-paths</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L24"/>
       <x:c r="M24" t="str">
-        <x:v>`write()` and `readlines()` on a manually opened file</x:v>
+        <x:v>Replace `loads` with `dumps`.</x:v>
       </x:c>
       <x:c r="N24" t="str">
-        <x:v>`write_text()` and `read_text()`</x:v>
+        <x:v>Replace the file mode with `"a"`.</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>`dump()` and `load()`</x:v>
+        <x:v>Convert the file object to `str(file)`.</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>`writerow()` and `reader()`</x:v>
+        <x:v>Use `json.load(file)` instead.</x:v>
       </x:c>
       <x:c r="Q24" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A25" t="str">
         <x:v>Python - MCQ - 11.3.4</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>Before reading an optional daily log, a script asks whether the path is present. Which method performs that check?</x:v>
+        <x:v>Check for an optional file before opening it
+A report may not have been generated yet. The script should test for it before attempting a read.
+```python
+from pathlib import Path
+report = Path("daily.txt")
+if ________:
+    text = report.read_text(encoding="utf-8")
+```
+Which condition fills the blank?</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>`Path.exists()` returns whether the referenced file or folder currently exists, allowing a simple conditional guard.</x:v>
+        <x:v>`Path.exists()` checks whether the target is present without opening it.</x:v>
       </x:c>
       <x:c r="D25" t="n">
         <x:v>1</x:v>
@@ -1619,7 +1694,7 @@
         <x:v>easy</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>understand</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H25" t="str">
         <x:v>python - Set 3</x:v>
@@ -1635,30 +1710,32 @@
       </x:c>
       <x:c r="L25"/>
       <x:c r="M25" t="str">
-        <x:v>`Path.read()`</x:v>
+        <x:v>`report.is_dir()`</x:v>
       </x:c>
       <x:c r="N25" t="str">
-        <x:v>`Path.opened()`</x:v>
+        <x:v>`report.exists()`</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>`Path.available()`</x:v>
+        <x:v>`report.parent.exists()`</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>`Path.exists()`</x:v>
+        <x:v>`bool(report.name)`</x:v>
       </x:c>
       <x:c r="Q25" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="66" hidden="0" customHeight="1">
       <x:c r="A26" t="str">
         <x:v>Python - MCQ - 11.3.5</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>A reports folder contains `day1.csv`, `day2.csv`, and `notes.txt`. Which pattern selects exactly the CSV files in that folder?</x:v>
+        <x:v>Predict the first failure when reading a missing path
+A script assumes `day4.txt` exists and opens it in read mode, but the file has never been created.
+Which execution account is correct?</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>`*.csv` accepts any filename prefix but requires the `.csv` suffix, so the TXT note is excluded.</x:v>
+        <x:v>Read mode requires an existing file; it does not create one.</x:v>
       </x:c>
       <x:c r="D26" t="n">
         <x:v>1</x:v>
@@ -1682,34 +1759,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>glob-pattern-matching</x:v>
+        <x:v>file-errors</x:v>
       </x:c>
       <x:c r="L26"/>
       <x:c r="M26" t="str">
-        <x:v>`day*.txt`</x:v>
+        <x:v>`open("day4.txt", "r")` raises `FileNotFoundError` immediately.</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>`**/*.txt`</x:v>
+        <x:v>Read mode creates an empty file and returns an empty string.</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>`*.csv`</x:v>
+        <x:v>Python silently changes the mode to append.</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>`csv.*`</x:v>
+        <x:v>The failure occurs only when the program later closes the file.</x:v>
       </x:c>
       <x:c r="Q26" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="66" hidden="0" customHeight="1">
       <x:c r="A27" t="str">
         <x:v>Python - MCQ - 11.3.6</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>A data folder contains text files both at its top level and inside nested subfolders. Which Path glob searches every level?</x:v>
+        <x:v>Keep text encoding consistent across machines
+A receipt containing `₹` is written on one operating system and read on another. The two operations must agree on character encoding.
+Which practice gives the clearest portable contract?</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>The double asterisk crosses directory levels. `**/*.txt` finds text files directly inside the starting folder and beneath its subfolders.</x:v>
+        <x:v>Explicit UTF-8 makes both operations use the same broad, predictable character mapping.</x:v>
       </x:c>
       <x:c r="D27" t="n">
         <x:v>1</x:v>
@@ -1721,7 +1800,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G27" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H27" t="str">
         <x:v>python - Set 3</x:v>
@@ -1733,34 +1812,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>glob-pattern-matching</x:v>
+        <x:v>file-errors</x:v>
       </x:c>
       <x:c r="L27"/>
       <x:c r="M27" t="str">
-        <x:v>`**/*.txt`</x:v>
+        <x:v>Use the system default on writing and guess on reading.</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>`*.txt` only</x:v>
+        <x:v>Remove the symbol before writing.</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>`txt/**`</x:v>
+        <x:v>Use UTF-8 explicitly for both operations.</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>`*/.txt`</x:v>
+        <x:v>Open the text file in CSV mode.</x:v>
       </x:c>
       <x:c r="Q27" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="66" hidden="0" customHeight="1">
       <x:c r="A28" t="str">
         <x:v>Python - MCQ - 11.3.7</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>A developer switches from `glob.glob(pattern)` to `Path(folder).glob(pattern)`. What important result-type difference should the code expect?</x:v>
+        <x:v>Extend a log across repeated program runs
+Each run of a scanner should add one new wristband ID while keeping every ID written by earlier runs.
+Which mode should the scanner use?</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>The standalone function returns matching path strings. `Path.glob()` integrates with pathlib and yields Path objects.</x:v>
+        <x:v>Append mode writes at the end of an existing file and creates it when absent.</x:v>
       </x:c>
       <x:c r="D28" t="n">
         <x:v>1</x:v>
@@ -1769,10 +1850,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F28" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G28" t="str">
-        <x:v>understand</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H28" t="str">
         <x:v>python - Set 3</x:v>
@@ -1784,34 +1865,42 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>glob-pattern-matching</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L28"/>
       <x:c r="M28" t="str">
-        <x:v>Both always return open file objects</x:v>
+        <x:v>`"r"`</x:v>
       </x:c>
       <x:c r="N28" t="str">
-        <x:v>`Path.glob()` returns only folder names</x:v>
+        <x:v>`"a"`</x:v>
       </x:c>
       <x:c r="O28" t="str">
-        <x:v>`glob.glob()` returns dictionaries</x:v>
+        <x:v>`"w"`</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>`Path.glob()` yields Path objects while `glob.glob()` returns strings</x:v>
+        <x:v>No mode, because every mode appends</x:v>
       </x:c>
       <x:c r="Q28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A29" t="str">
         <x:v>Python - MCQ - 11.3.8</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>A script hard-codes three sales filenames. A fourth daily file is later added and silently ignored. Why is a glob pattern a better design?</x:v>
+        <x:v>Account for a crash inside a managed write
+A report writes one line, encounters an unrelated division-by-zero error, and has a second write below the failing line.
+```python
+with open("report.txt", "w", encoding="utf-8") as file:
+    file.write("Before\n")
+    value = 10 / 0
+    file.write("After\n")
+```
+Which account best describes the file-handling behaviour?</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>A glob describes the filename shape rather than a fixed list. New files matching that shape are discovered without changing the code.</x:v>
+        <x:v>A context manager guarantees cleanup but does not suppress this error or execute skipped statements.</x:v>
       </x:c>
       <x:c r="D29" t="n">
         <x:v>1</x:v>
@@ -1820,10 +1909,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G29" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H29" t="str">
         <x:v>python - Set 3</x:v>
@@ -1835,34 +1924,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K29" t="str">
-        <x:v>glob-pattern-matching</x:v>
+        <x:v>context-managed-files</x:v>
       </x:c>
       <x:c r="L29"/>
       <x:c r="M29" t="str">
-        <x:v>It converts every file to JSON</x:v>
+        <x:v>The error is suppressed, and both lines are written.</x:v>
       </x:c>
       <x:c r="N29" t="str">
-        <x:v>It discovers newly added files that match the stated pattern</x:v>
+        <x:v>The file remains open because the block did not finish normally.</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>It guarantees files contain valid data</x:v>
+        <x:v>The second write runs during automatic cleanup.</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>It sorts file contents automatically</x:v>
+        <x:v>Error propagates; the file closes; the second write is skipped.</x:v>
       </x:c>
       <x:c r="Q29" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="66" hidden="0" customHeight="1">
       <x:c r="A30" t="str">
         <x:v>Python - MCQ - 11.3.9</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>A CSV row contains quantity `'2'` and price `'350'`. The code uses `row['quantity'] * row['price']`. What correction is required for revenue arithmetic?</x:v>
+        <x:v>Choose between CSV and JSON from the data shape
+Dataset A is a flat table of sales rows. Dataset B is a dictionary of stalls, each containing its own item dictionary.
+Which pairing is most suitable?</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>CSV readers return fields as strings. Both numeric fields must be converted, such as with `int(...)`, before multiplying them.</x:v>
+        <x:v>CSV fits flat rows and columns, while JSON naturally preserves nested structure.</x:v>
       </x:c>
       <x:c r="D30" t="n">
         <x:v>1</x:v>
@@ -1871,10 +1962,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F30" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G30" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H30" t="str">
         <x:v>python - Set 3</x:v>
@@ -1886,34 +1977,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>csv-processing</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L30"/>
       <x:c r="M30" t="str">
-        <x:v>Convert both fields to numbers before multiplication</x:v>
+        <x:v>JSON for A only; plain variables for B</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>Use `strip()` on only the price</x:v>
+        <x:v>CSV for both because all files are text</x:v>
       </x:c>
       <x:c r="O30" t="str">
-        <x:v>Replace DictReader with JSON dump</x:v>
+        <x:v>CSV for A and JSON for B</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>Open the CSV in append mode</x:v>
+        <x:v>JSON for A and CSV for B because nesting belongs in columns</x:v>
       </x:c>
       <x:c r="Q30" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="66" hidden="0" customHeight="1">
       <x:c r="A31" t="str">
         <x:v>Python - MCQ - 11.3.10</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>A list of sales dictionaries must be written with columns in the order item, quantity, price. Which writer setup provides named-column control?</x:v>
+        <x:v>Create a reports folder safely on repeated runs
+A startup step may run many times. It should create `reports/` when absent and do nothing harmful when the folder already exists.
+Which statement matches that requirement?</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>`csv.DictWriter` accepts `fieldnames` to define the CSV column order. `writeheader()` then writes those names as the header row.</x:v>
+        <x:v>`mkdir(exist_ok=True)` creates the directory or leaves the existing one in place without an error.</x:v>
       </x:c>
       <x:c r="D31" t="n">
         <x:v>1</x:v>
@@ -1937,34 +2030,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>csv-processing</x:v>
+        <x:v>file-paths</x:v>
       </x:c>
       <x:c r="L31"/>
       <x:c r="M31" t="str">
-        <x:v>`csv.reader(file)`</x:v>
+        <x:v>`Path("reports").mkdir(exist_ok=True)`</x:v>
       </x:c>
       <x:c r="N31" t="str">
-        <x:v>`csv.DictWriter(file, fieldnames=['item', 'quantity', 'price'])`</x:v>
+        <x:v>`Path("reports").mkdir(exist_ok=False)`</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>`json.DictWriter(file, fieldnames=['item', 'quantity', 'price'])` as a CSV substitute</x:v>
+        <x:v>`Path("reports").touch(exist_ok=True)`</x:v>
       </x:c>
       <x:c r="P31" t="str">
-        <x:v>`file.readlines(fieldnames)`</x:v>
+        <x:v>`Path("reports").parent.mkdir(exist_ok=True)`</x:v>
       </x:c>
       <x:c r="Q31" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="66" hidden="0" customHeight="1">
       <x:c r="A32" t="str">
         <x:v>Python - MCQ - 11.4.1</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>A `DictWriter` writes data rows correctly, but the resulting file has no header. Which call was most likely omitted?</x:v>
+        <x:v>Account for the result type of two glob interfaces
+One implementation uses `Path("reports").glob("*.csv")`; another uses `glob.glob("reports/*.csv")`. Later code depends on whether results are path objects or strings.
+Which comparison is accurate?</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>Creating a DictWriter does not automatically emit the header. Calling `writer.writeheader()` writes the field names once before the data rows.</x:v>
+        <x:v>The two interfaces match similar patterns but represent their matched locations differently.</x:v>
       </x:c>
       <x:c r="D32" t="n">
         <x:v>1</x:v>
@@ -1976,7 +2071,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G32" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H32" t="str">
         <x:v>python - Set 4</x:v>
@@ -1988,34 +2083,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K32" t="str">
-        <x:v>csv-processing</x:v>
+        <x:v>glob-pattern-matching</x:v>
       </x:c>
       <x:c r="L32"/>
       <x:c r="M32" t="str">
-        <x:v>`writer.writerow([])`</x:v>
+        <x:v>Both return file contents instead of names.</x:v>
       </x:c>
       <x:c r="N32" t="str">
-        <x:v>`writer.readheader()`</x:v>
+        <x:v>`Path.glob()` yields `Path`; `glob.glob()` yields strings.</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>`file.header = True` before writing all rows</x:v>
+        <x:v>`glob.glob()` returns dictionaries keyed by extension.</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>`writer.writeheader()`</x:v>
+        <x:v>`Path.glob()` opens every matching file automatically.</x:v>
       </x:c>
       <x:c r="Q32" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="66" hidden="0" customHeight="1">
       <x:c r="A33" t="str">
         <x:v>Python - MCQ - 11.4.2</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>A developer has an open JSON file and also a JSON-formatted string. Which pairing reads both into Python objects correctly?</x:v>
+        <x:v>Choose the filename that defeats a numeric assumption
+A developer assumes `day*_sales.txt` selects only filenames whose middle section is a day number. A test must demonstrate that `*` is not a numeric validator.
+Which additional filename is the clearest counterexample?</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>`json.load(file)` reads from an open file object, while `json.loads(text)` parses a JSON string. The `s` form is the string form.</x:v>
+        <x:v>`day_final_sales.txt` satisfies the literal prefix and suffix because `*` accepts `final` just as readily as digits.</x:v>
       </x:c>
       <x:c r="D33" t="n">
         <x:v>1</x:v>
@@ -2027,7 +2124,7 @@
         <x:v>hard</x:v>
       </x:c>
       <x:c r="G33" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H33" t="str">
         <x:v>python - Set 4</x:v>
@@ -2039,34 +2136,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K33" t="str">
-        <x:v>json-processing</x:v>
+        <x:v>glob-pattern-matching</x:v>
       </x:c>
       <x:c r="L33"/>
       <x:c r="M33" t="str">
-        <x:v>Use `loads` for both inputs</x:v>
+        <x:v>`day1_sales.csv`</x:v>
       </x:c>
       <x:c r="N33" t="str">
-        <x:v>Use `dump` for the file and `dumps` for the string</x:v>
+        <x:v>`week1_sales.txt`</x:v>
       </x:c>
       <x:c r="O33" t="str">
-        <x:v>Use `json.load(file)` and `json.loads(text)`</x:v>
+        <x:v>`day2_summary.txt`</x:v>
       </x:c>
       <x:c r="P33" t="str">
-        <x:v>Use `readlines()` for both</x:v>
+        <x:v>`day_final_sales.txt`</x:v>
       </x:c>
       <x:c r="Q33" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="66" hidden="0" customHeight="1">
       <x:c r="A34" t="str">
         <x:v>Python - MCQ - 11.4.3</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>A program needs JSON text in memory to send elsewhere, not a JSON file on disk. Which function returns a string?</x:v>
+        <x:v>Make a saved JSON report readable to humans
+A nested JSON file will be inspected manually during an audit, so it should use readable line breaks and indentation.
+Which argument supplies that formatting during `json.dump`?</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>`json.dumps(object)` serializes a Python object to a JSON string. `json.dump` instead writes to an open file.</x:v>
+        <x:v>The optional `indent` argument pretty-prints nested JSON without changing its data.</x:v>
       </x:c>
       <x:c r="D34" t="n">
         <x:v>1</x:v>
@@ -2075,10 +2174,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F34" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G34" t="str">
-        <x:v>understand</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H34" t="str">
         <x:v>python - Set 4</x:v>
@@ -2094,30 +2193,36 @@
       </x:c>
       <x:c r="L34"/>
       <x:c r="M34" t="str">
-        <x:v>`json.load()`</x:v>
+        <x:v>`indent=4`</x:v>
       </x:c>
       <x:c r="N34" t="str">
-        <x:v>`json.dumps()`</x:v>
+        <x:v>`newline=""`</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>`csv.writer()`</x:v>
+        <x:v>`mode="pretty"`</x:v>
       </x:c>
       <x:c r="P34" t="str">
-        <x:v>`Path.write_text()`</x:v>
+        <x:v>`fieldnames=4`</x:v>
       </x:c>
       <x:c r="Q34" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="132" hidden="0" customHeight="1">
       <x:c r="A35" t="str">
         <x:v>Python - MCQ - 11.4.4</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>A Python tuple is serialized to JSON and then loaded again. Which limitation matters if the program must preserve tuple identity?</x:v>
+        <x:v>Replace an entire small text report through a Path
+A short summary file should contain exactly the newest report text. No line-by-line processing or append behaviour is needed.
+```python
+from pathlib import Path
+report = Path("summary.txt")
+```
+Which operation directly writes the complete text?</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>JSON has arrays but no distinct tuple type. A Python tuple is saved as a JSON array and loads back as a list, so the distinction is lost.</x:v>
+        <x:v>`Path.write_text` writes an entire text value directly to the target path.</x:v>
       </x:c>
       <x:c r="D35" t="n">
         <x:v>1</x:v>
@@ -2126,10 +2231,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F35" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G35" t="str">
-        <x:v>analyze</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H35" t="str">
         <x:v>python - Set 4</x:v>
@@ -2141,34 +2246,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>json-processing</x:v>
+        <x:v>file-paths</x:v>
       </x:c>
       <x:c r="L35"/>
       <x:c r="M35" t="str">
-        <x:v>The tuple becomes a JSON array and loads back as a list</x:v>
+        <x:v>`report.touch()` followed by `report.open()` with no write</x:v>
       </x:c>
       <x:c r="N35" t="str">
-        <x:v>JSON refuses all sequences</x:v>
+        <x:v>`report.read_text(encoding="utf-8")`</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>The tuple becomes a CSV row</x:v>
+        <x:v>`report.write_text("Ready", encoding="utf-8")`</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>Only the first tuple item is saved</x:v>
+        <x:v>`report.rename("Ready")`</x:v>
       </x:c>
       <x:c r="Q35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="66" hidden="0" customHeight="1">
       <x:c r="A36" t="str">
         <x:v>Python - MCQ - 11.4.5</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>A project must store flat student rows for spreadsheet exchange and a nested application configuration. Which format choice best matches both shapes?</x:v>
+        <x:v>Prevent platform-specific blank lines in a CSV export
+A CSV writer produces extra blank rows on one teammate's operating system. The file was opened without the CSV-specific newline setting.
+Which opening style follows the lesson's recommended habit?</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>CSV suits flat rows and columns, while JSON naturally represents nested dictionaries and lists. Choosing by data shape avoids awkward manual encoding.</x:v>
+        <x:v>`newline=""` lets the CSV module manage row endings consistently across platforms.</x:v>
       </x:c>
       <x:c r="D36" t="n">
         <x:v>1</x:v>
@@ -2177,7 +2284,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F36" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G36" t="str">
         <x:v>analyze</x:v>
@@ -2192,34 +2299,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K36" t="str">
-        <x:v>json-processing</x:v>
+        <x:v>csv-processing</x:v>
       </x:c>
       <x:c r="L36"/>
       <x:c r="M36" t="str">
-        <x:v>Use CSV for both because it preserves all nested types</x:v>
+        <x:v>`open("sales.csv", "r")`</x:v>
       </x:c>
       <x:c r="N36" t="str">
-        <x:v>Use JSON for the rows and plain text for the configuration</x:v>
+        <x:v>`open("sales.csv", "w", newline="\n", encoding="utf-8")`</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>Use CSV for the student table and JSON for the nested configuration</x:v>
+        <x:v>`open("sales.csv", "a", encoding=None)`</x:v>
       </x:c>
       <x:c r="P36" t="str">
-        <x:v>Use glob patterns as the storage format</x:v>
+        <x:v>`open("sales.csv", "w", newline="", encoding="utf-8")`</x:v>
       </x:c>
       <x:c r="Q36" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="66" hidden="0" customHeight="1">
       <x:c r="A37" t="str">
         <x:v>Python - MCQ - 11.4.6</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>A script opens `missing.txt` in read mode without checking whether it exists. What failure should the developer expect?</x:v>
+        <x:v>Decide whether two complete-reading implementations are equivalent
+For an existing, small UTF-8 text file, Version A uses a managed `open` call and `read()`. Version B uses `Path.read_text` with the same encoding. Neither implementation needs streaming or access to the open file object.
+Which review conclusion is accurate?</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>Read mode requires an existing file. If the path does not exist, `open` raises `FileNotFoundError` immediately.</x:v>
+        <x:v>Under the stated constraints, both implementations read the entire decoded text into one string and release the file resource; they differ mainly in interface.</x:v>
       </x:c>
       <x:c r="D37" t="n">
         <x:v>1</x:v>
@@ -2228,10 +2337,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F37" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H37" t="str">
         <x:v>python - Set 4</x:v>
@@ -2243,34 +2352,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>file-errors</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L37"/>
       <x:c r="M37" t="str">
-        <x:v>An empty file is always created</x:v>
+        <x:v>Version A returns a list of lines, while Version B returns bytes.</x:v>
       </x:c>
       <x:c r="N37" t="str">
-        <x:v>The read returns an empty string</x:v>
+        <x:v>Equivalent here: both return all text and close the file.</x:v>
       </x:c>
       <x:c r="O37" t="str">
-        <x:v>The path changes to the current folder</x:v>
+        <x:v>Version B necessarily appends an extra newline to the returned text.</x:v>
       </x:c>
       <x:c r="P37" t="str">
-        <x:v>A FileNotFoundError is raised</x:v>
+        <x:v>Version A leaves the file open after its `with` block.</x:v>
       </x:c>
       <x:c r="Q37" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="66" hidden="0" customHeight="1">
       <x:c r="A38" t="str">
         <x:v>Python - MCQ - 11.4.7</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>A receipt containing `₹1500` must be written on one machine and read correctly on another. Which habit removes reliance on system-default encodings?</x:v>
+        <x:v>Design a restart-safe attendee tracker
+An attendee tracker must preserve IDs after shutdown, load them when the next run begins, and add later scans without erasing earlier ones.
+Which workflow satisfies all three needs?</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>Explicitly using UTF-8 for both operations ensures the writer and reader interpret the same bytes as the same characters.</x:v>
+        <x:v>Reading restores persistent state, and append mode extends the stored history non-destructively.</x:v>
       </x:c>
       <x:c r="D38" t="n">
         <x:v>1</x:v>
@@ -2282,7 +2393,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>apply</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H38" t="str">
         <x:v>python - Set 4</x:v>
@@ -2294,34 +2405,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>file-errors</x:v>
+        <x:v>file-operations</x:v>
       </x:c>
       <x:c r="L38"/>
       <x:c r="M38" t="str">
-        <x:v>Specify `encoding='utf-8'` on both the write and read</x:v>
+        <x:v>Store IDs only in a set and print it before exit.</x:v>
       </x:c>
       <x:c r="N38" t="str">
-        <x:v>Use different encodings for each machine</x:v>
+        <x:v>Open the log in write mode for every scan.</x:v>
       </x:c>
       <x:c r="O38" t="str">
-        <x:v>Remove the file extension</x:v>
+        <x:v>Load saved IDs at startup and append later scans.</x:v>
       </x:c>
       <x:c r="P38" t="str">
-        <x:v>Open the file twice in write mode</x:v>
+        <x:v>Recreate an empty variable at the start of every run.</x:v>
       </x:c>
       <x:c r="Q38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="66" hidden="0" customHeight="1">
       <x:c r="A39" t="str">
         <x:v>Python - MCQ - 11.4.8</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>A CSV analyzer computes average CGPA from `DictReader` rows but receives a TypeError while adding values. Which repair addresses the data-model issue without changing the file?</x:v>
+        <x:v>Write dictionary rows with matching CSV columns
+A CSV export already has a `DictWriter` configured with `fieldnames`, has written its header, and now holds a list named `sales` containing dictionaries.
+Which call writes every dictionary as a row?</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>DictReader supplies CSV fields as strings. Converting each valid `row['cgpa']` to `float` before accumulation makes the average numeric; validation of missing values can be added around that conversion later.</x:v>
+        <x:v>`DictWriter.writerows` maps each dictionary's keys to the configured CSV fields.</x:v>
       </x:c>
       <x:c r="D39" t="n">
         <x:v>1</x:v>
@@ -2330,10 +2443,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>analyze</x:v>
+        <x:v>apply</x:v>
       </x:c>
       <x:c r="H39" t="str">
         <x:v>python - Set 4</x:v>
@@ -2349,30 +2462,32 @@
       </x:c>
       <x:c r="L39"/>
       <x:c r="M39" t="str">
-        <x:v>Use append mode when opening the CSV</x:v>
+        <x:v>`writer.writerows(sales)`</x:v>
       </x:c>
       <x:c r="N39" t="str">
-        <x:v>Convert each CGPA string to `float` before summing</x:v>
+        <x:v>`writer.writerow(sales)`</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>Serialize every row to JSON before reading it</x:v>
+        <x:v>`writer.writeheader()`</x:v>
       </x:c>
       <x:c r="P39" t="str">
-        <x:v>Replace the header with numeric column indexes</x:v>
+        <x:v>`writer.writerows(sales[0])`</x:v>
       </x:c>
       <x:c r="Q39" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="66" hidden="0" customHeight="1">
       <x:c r="A40" t="str">
         <x:v>Python - MCQ - 11.4.9</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>A developer writes `open('notes.txt')` without a mode argument. Which mode does Python use by default?</x:v>
+        <x:v>Reject a format that cannot naturally preserve nesting
+A configuration contains dictionaries inside dictionaries, lists, numbers, booleans, and `None`. A proposed CSV export would flatten everything into manually encoded cells.
+Which design judgment is strongest?</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>The default mode for `open()` is read mode. The file must already exist, just as if the caller had written `open('notes.txt', 'r')`.</x:v>
+        <x:v>JSON models nested structured values directly, while CSV fundamentally represents rows and columns of text.</x:v>
       </x:c>
       <x:c r="D40" t="n">
         <x:v>1</x:v>
@@ -2381,10 +2496,10 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F40" t="str">
-        <x:v>easy</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G40" t="str">
-        <x:v>understand</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H40" t="str">
         <x:v>python - Set 4</x:v>
@@ -2396,34 +2511,36 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K40" t="str">
-        <x:v>file-operations</x:v>
+        <x:v>json-processing</x:v>
       </x:c>
       <x:c r="L40"/>
       <x:c r="M40" t="str">
-        <x:v>Append mode</x:v>
+        <x:v>CSV automatically reconstructs arbitrary nesting and Python types.</x:v>
       </x:c>
       <x:c r="N40" t="str">
-        <x:v>Write mode</x:v>
+        <x:v>Plain `split(",")` preserves nested objects better than both modules.</x:v>
       </x:c>
       <x:c r="O40" t="str">
-        <x:v>Read mode</x:v>
+        <x:v>Both formats preserve tuples as tuples with no special handling.</x:v>
       </x:c>
       <x:c r="P40" t="str">
-        <x:v>Binary write mode</x:v>
+        <x:v>Use JSON for the nesting; CSV would require custom flattening.</x:v>
       </x:c>
       <x:c r="Q40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="66" hidden="0" customHeight="1">
       <x:c r="A41" t="str">
         <x:v>Python - MCQ - 11.4.10</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>For `Path('reports/day1_sales.csv')`, a dashboard needs the containing folder rather than the filename or extension. Which property returns it?</x:v>
+        <x:v>Assemble a reliable daily-report pipeline
+A festival pipeline must create a reports folder safely, append text logs, export flat sales rows, save a nested summary, and tolerate a report that has not yet been generated.
+Which design best applies the full unit?</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>The `.parent` property returns the containing path, which is `reports` here. `.name`, `.stem`, and `.suffix` describe the final filename instead.</x:v>
+        <x:v>The design selects the safe path, mode, context management, format, and missing-file guard appropriate to each requirement.</x:v>
       </x:c>
       <x:c r="D41" t="n">
         <x:v>1</x:v>
@@ -2435,7 +2552,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="G41" t="str">
-        <x:v>apply</x:v>
+        <x:v>evaluate</x:v>
       </x:c>
       <x:c r="H41" t="str">
         <x:v>python - Set 4</x:v>
@@ -2447,23 +2564,23 @@
         <x:v>file-handling</x:v>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>file-paths</x:v>
+        <x:v>file-errors</x:v>
       </x:c>
       <x:c r="L41"/>
       <x:c r="M41" t="str">
-        <x:v>The `.name` property for the complete final filename</x:v>
+        <x:v>Build paths by string guessing, use write mode for every log entry, and parse all data with `split(",")`.</x:v>
       </x:c>
       <x:c r="N41" t="str">
-        <x:v>`.stem`</x:v>
+        <x:v>Use `Path`, `with`, append logs, CSV, JSON, and guarded reads.</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>`.suffix`</x:v>
+        <x:v>Keep everything only in variables and rely on program memory after restart.</x:v>
       </x:c>
       <x:c r="P41" t="str">
-        <x:v>`.parent`</x:v>
+        <x:v>Upload open file objects so another machine can continue using them.</x:v>
       </x:c>
       <x:c r="Q41" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>